<commit_message>
fix: correct JPA method name for composite key lookup
The method `findByPharmacyIdAndDrugId` was incorrectly named for JPA's derived query when Pharmacy and Drug have composite keys. Updated to `findByPharmacyId_IDAndDrugId_ID` to properly resolve the nested ID fields. Also fixed missing newlines at end of files and updated the drugs template.
</commit_message>
<xml_diff>
--- a/server/drugs_template.xlsx
+++ b/server/drugs_template.xlsx
@@ -17,20 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-    </font>
-    <font>
-      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="2">
@@ -53,10 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -424,111 +415,104 @@
   </sheetPr>
   <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>quantity</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>pharmacy_name</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>city</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>region</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Paracetamol</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n">
+      <c r="B2" t="n">
         <v>100</v>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Main Street Pharmacy</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Douala</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Littoral</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Ibuprofen</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n">
+      <c r="B3" t="n">
         <v>50</v>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Main Street Pharmacy</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Douala</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Littoral</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Amoxicillin</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n">
+      <c r="B4" t="n">
         <v>200</v>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Main Street Pharmacy</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Douala</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Littoral</t>
         </is>

</xml_diff>